<commit_message>
Trước defend để có gì sau cần xem lại thì xem (chuẩn bị chỉnh sửa code)
</commit_message>
<xml_diff>
--- a/initial solution/rule-based-final/small_scale_v2 copy/multi_seed_results.xlsx
+++ b/initial solution/rule-based-final/small_scale_v2 copy/multi_seed_results.xlsx
@@ -473,19 +473,19 @@
         <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>87715.94888630357</v>
+        <v>90073.94888630357</v>
       </c>
       <c r="D2" t="n">
-        <v>87715.94888630357</v>
+        <v>89503.94888630357</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>570</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.6328133795038633</v>
       </c>
       <c r="G2" t="n">
-        <v>325.4605934619904</v>
+        <v>180.0603830814362</v>
       </c>
     </row>
     <row r="3">
@@ -496,19 +496,19 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>83909.90826016715</v>
+        <v>86081.90826016715</v>
       </c>
       <c r="D3" t="n">
-        <v>83909.90826016715</v>
+        <v>85591.90826016715</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>490</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>0.569225299373084</v>
       </c>
       <c r="G3" t="n">
-        <v>213.8100469112396</v>
+        <v>128.7974088191986</v>
       </c>
     </row>
     <row r="4">
@@ -519,19 +519,19 @@
         <v>28</v>
       </c>
       <c r="C4" t="n">
-        <v>129283.9436782268</v>
+        <v>153120.4436782268</v>
       </c>
       <c r="D4" t="n">
-        <v>129283.9436782268</v>
+        <v>130922.4436782268</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>22198</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>14.49708443024613</v>
       </c>
       <c r="G4" t="n">
-        <v>671.5911540985107</v>
+        <v>258.5204303264618</v>
       </c>
     </row>
     <row r="5">
@@ -542,19 +542,19 @@
         <v>23</v>
       </c>
       <c r="C5" t="n">
-        <v>65121.00165811017</v>
+        <v>109361.0016581102</v>
       </c>
       <c r="D5" t="n">
-        <v>65121.00165811017</v>
+        <v>67688.00165811017</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>41673</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>38.10590554965857</v>
       </c>
       <c r="G5" t="n">
-        <v>494.8854413032532</v>
+        <v>237.4926371574402</v>
       </c>
     </row>
     <row r="6">
@@ -565,19 +565,19 @@
         <v>21</v>
       </c>
       <c r="C6" t="n">
-        <v>115730.9328035403</v>
+        <v>131099.4328035403</v>
       </c>
       <c r="D6" t="n">
-        <v>115730.9328035403</v>
+        <v>129055.9328035403</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>2043.499999999985</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1.558740534798715</v>
       </c>
       <c r="G6" t="n">
-        <v>519.4485812187195</v>
+        <v>251.1403541564941</v>
       </c>
     </row>
     <row r="7">
@@ -588,19 +588,19 @@
         <v>19</v>
       </c>
       <c r="C7" t="n">
-        <v>140158.9154637347</v>
+        <v>182670.4154637347</v>
       </c>
       <c r="D7" t="n">
-        <v>140158.9154637347</v>
+        <v>143493.9154637347</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>39176.5</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>21.44654891189956</v>
       </c>
       <c r="G7" t="n">
-        <v>474.6115329265594</v>
+        <v>308.9598631858826</v>
       </c>
     </row>
     <row r="8">
@@ -611,19 +611,19 @@
         <v>29</v>
       </c>
       <c r="C8" t="n">
-        <v>158898.3047248611</v>
+        <v>195497.2047248611</v>
       </c>
       <c r="D8" t="n">
-        <v>158898.3047248611</v>
+        <v>161535.3047248611</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>33961.89999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>17.37206424398615</v>
       </c>
       <c r="G8" t="n">
-        <v>703.5186533927917</v>
+        <v>382.9775457382202</v>
       </c>
     </row>
     <row r="9">
@@ -634,19 +634,19 @@
         <v>28</v>
       </c>
       <c r="C9" t="n">
-        <v>136353.01893729</v>
+        <v>160508.51893729</v>
       </c>
       <c r="D9" t="n">
-        <v>136353.01893729</v>
+        <v>138797.51893729</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>21711</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>13.52638485716911</v>
       </c>
       <c r="G9" t="n">
-        <v>489.2177634239197</v>
+        <v>434.1966483592987</v>
       </c>
     </row>
     <row r="10">
@@ -657,19 +657,19 @@
         <v>17</v>
       </c>
       <c r="C10" t="n">
-        <v>84964.1261748253</v>
+        <v>99550.1261748253</v>
       </c>
       <c r="D10" t="n">
-        <v>84964.1261748253</v>
+        <v>86635.1261748253</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>12915</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>12.97336376783619</v>
       </c>
       <c r="G10" t="n">
-        <v>321.2015950679779</v>
+        <v>192.836222410202</v>
       </c>
     </row>
     <row r="11">
@@ -680,19 +680,19 @@
         <v>25</v>
       </c>
       <c r="C11" t="n">
-        <v>159861.8006172027</v>
+        <v>235570.3006172027</v>
       </c>
       <c r="D11" t="n">
-        <v>159861.8006172027</v>
+        <v>161931.8006172027</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>73638.5</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>31.25967059814606</v>
       </c>
       <c r="G11" t="n">
-        <v>493.5540504455566</v>
+        <v>345.4401528835297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>